<commit_message>
Första semi + stavningsfel
</commit_message>
<xml_diff>
--- a/Resultat.xlsx
+++ b/Resultat.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ellabacklund/Claude_project/vm-tippning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A143259-78D9-CC40-AD2D-6B3A04A7EBDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5F114B-88EC-0145-A2CA-1947098EB5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15880" xr2:uid="{F9B9E0B2-0622-234A-8FBC-8B192F70E9B7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>Frankrike</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>Argentina</t>
+  </si>
+  <si>
+    <t>Schweiz</t>
   </si>
 </sst>
 </file>
@@ -538,7 +541,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -589,7 +592,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>